<commit_message>
Daily recap, matchup updates, learning and research 2026-08-16
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-16.xlsx
+++ b/data/k-props/2026-08-16.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="98">
   <si>
     <t>date</t>
   </si>
@@ -145,28 +145,40 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>&lt;6</t>
+  </si>
+  <si>
+    <t>Freddy Peralta</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>Patrick Sandoval</t>
+  </si>
+  <si>
+    <t>Boston Red Sox @ Pittsburgh Pirates</t>
+  </si>
+  <si>
+    <t>&gt;=7</t>
+  </si>
+  <si>
+    <t>Lake Bachar</t>
+  </si>
+  <si>
+    <t>Opener / bullpen game</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t>&lt;6</t>
-  </si>
-  <si>
-    <t>Freddy Peralta</t>
-  </si>
-  <si>
-    <t>Patrick Sandoval</t>
-  </si>
-  <si>
-    <t>Boston Red Sox @ Pittsburgh Pirates</t>
-  </si>
-  <si>
-    <t>&gt;=7</t>
-  </si>
-  <si>
-    <t>Lake Bachar</t>
-  </si>
-  <si>
-    <t>Opener / bullpen game</t>
   </si>
   <si>
     <t>Michael Soroka</t>
@@ -874,17 +886,23 @@
       <c r="Y2">
         <v>0.88</v>
       </c>
+      <c r="Z2">
+        <v>6</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>-1.28</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>3.22</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.2245</v>
@@ -894,6 +912,18 @@
       </c>
       <c r="AH2">
         <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>2.78</v>
+      </c>
+      <c r="AJ2">
+        <v>2.78</v>
+      </c>
+      <c r="AK2">
+        <v>2.78</v>
+      </c>
+      <c r="AL2">
+        <v>2.78</v>
       </c>
       <c r="AM2">
         <v>3.22</v>
@@ -904,7 +934,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>6.5</v>
@@ -975,17 +1005,23 @@
       <c r="Y3">
         <v>1.0287</v>
       </c>
+      <c r="Z3">
+        <v>2</v>
+      </c>
       <c r="AA3" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB3">
+        <v>-1.13</v>
       </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD3">
         <v>5.37</v>
       </c>
       <c r="AE3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF3">
         <v>0.2017</v>
@@ -995,6 +1031,18 @@
       </c>
       <c r="AH3">
         <v>0</v>
+      </c>
+      <c r="AI3">
+        <v>-3.37</v>
+      </c>
+      <c r="AJ3">
+        <v>3.37</v>
+      </c>
+      <c r="AK3">
+        <v>-3.37</v>
+      </c>
+      <c r="AL3">
+        <v>3.37</v>
       </c>
       <c r="AM3">
         <v>5.37</v>
@@ -1005,7 +1053,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C4">
         <v>4.5</v>
@@ -1017,7 +1065,7 @@
         <v>120</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G4">
         <v>823344</v>
@@ -1076,17 +1124,23 @@
       <c r="Y4">
         <v>1.1015</v>
       </c>
+      <c r="Z4">
+        <v>6</v>
+      </c>
       <c r="AA4" t="s">
         <v>44</v>
       </c>
+      <c r="AB4">
+        <v>1.9</v>
+      </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD4">
         <v>7.22</v>
       </c>
       <c r="AE4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="AF4">
         <v>0.2162</v>
@@ -1096,6 +1150,18 @@
       </c>
       <c r="AH4">
         <v>-0.82</v>
+      </c>
+      <c r="AI4">
+        <v>-1.22</v>
+      </c>
+      <c r="AJ4">
+        <v>1.22</v>
+      </c>
+      <c r="AK4">
+        <v>-0.4</v>
+      </c>
+      <c r="AL4">
+        <v>0.4</v>
       </c>
       <c r="AM4">
         <v>6.4</v>
@@ -1106,16 +1172,16 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G5">
         <v>823344</v>
       </c>
       <c r="H5" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="I5">
         <v>2.4</v>
@@ -1169,16 +1235,16 @@
         <v>0.9171</v>
       </c>
       <c r="AA5" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD5">
         <v>2.22</v>
       </c>
       <c r="AE5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF5">
         <v>0.2682</v>
@@ -1198,7 +1264,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C6">
         <v>4.5</v>
@@ -1210,7 +1276,7 @@
         <v>-110</v>
       </c>
       <c r="F6" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G6">
         <v>824880</v>
@@ -1269,17 +1335,23 @@
       <c r="Y6">
         <v>1.0284</v>
       </c>
+      <c r="Z6">
+        <v>5</v>
+      </c>
       <c r="AA6" t="s">
         <v>44</v>
       </c>
+      <c r="AB6">
+        <v>0.94</v>
+      </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD6">
         <v>5.44</v>
       </c>
       <c r="AE6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF6">
         <v>0.2337</v>
@@ -1289,6 +1361,18 @@
       </c>
       <c r="AH6">
         <v>0</v>
+      </c>
+      <c r="AI6">
+        <v>-0.44</v>
+      </c>
+      <c r="AJ6">
+        <v>0.44</v>
+      </c>
+      <c r="AK6">
+        <v>-0.44</v>
+      </c>
+      <c r="AL6">
+        <v>0.44</v>
       </c>
       <c r="AM6">
         <v>5.44</v>
@@ -1299,7 +1383,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C7">
         <v>3.5</v>
@@ -1311,7 +1395,7 @@
         <v>118</v>
       </c>
       <c r="F7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G7">
         <v>824880</v>
@@ -1370,17 +1454,23 @@
       <c r="Y7">
         <v>0.88</v>
       </c>
+      <c r="Z7">
+        <v>5</v>
+      </c>
       <c r="AA7" t="s">
         <v>44</v>
       </c>
+      <c r="AB7">
+        <v>-0.21</v>
+      </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD7">
         <v>3.29</v>
       </c>
       <c r="AE7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF7">
         <v>0.1926</v>
@@ -1390,6 +1480,18 @@
       </c>
       <c r="AH7">
         <v>0</v>
+      </c>
+      <c r="AI7">
+        <v>1.71</v>
+      </c>
+      <c r="AJ7">
+        <v>1.71</v>
+      </c>
+      <c r="AK7">
+        <v>1.71</v>
+      </c>
+      <c r="AL7">
+        <v>1.71</v>
       </c>
       <c r="AM7">
         <v>3.29</v>
@@ -1400,7 +1502,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C8">
         <v>4.5</v>
@@ -1412,7 +1514,7 @@
         <v>125</v>
       </c>
       <c r="F8" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G8">
         <v>822774</v>
@@ -1471,17 +1573,23 @@
       <c r="Y8">
         <v>0.9762</v>
       </c>
+      <c r="Z8">
+        <v>4</v>
+      </c>
       <c r="AA8" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB8">
+        <v>-0.07</v>
       </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD8">
         <v>4.43</v>
       </c>
       <c r="AE8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF8">
         <v>0.2377</v>
@@ -1491,6 +1599,18 @@
       </c>
       <c r="AH8">
         <v>0</v>
+      </c>
+      <c r="AI8">
+        <v>-0.43</v>
+      </c>
+      <c r="AJ8">
+        <v>0.43</v>
+      </c>
+      <c r="AK8">
+        <v>-0.43</v>
+      </c>
+      <c r="AL8">
+        <v>0.43</v>
       </c>
       <c r="AM8">
         <v>4.43</v>
@@ -1501,7 +1621,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C9">
         <v>8.5</v>
@@ -1513,7 +1633,7 @@
         <v>-110</v>
       </c>
       <c r="F9" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G9">
         <v>822774</v>
@@ -1572,17 +1692,23 @@
       <c r="Y9">
         <v>1.0285</v>
       </c>
+      <c r="Z9">
+        <v>10</v>
+      </c>
       <c r="AA9" t="s">
         <v>44</v>
       </c>
+      <c r="AB9">
+        <v>0.27</v>
+      </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD9">
         <v>9.59</v>
       </c>
       <c r="AE9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="AF9">
         <v>0.3641</v>
@@ -1592,6 +1718,18 @@
       </c>
       <c r="AH9">
         <v>-0.82</v>
+      </c>
+      <c r="AI9">
+        <v>0.41</v>
+      </c>
+      <c r="AJ9">
+        <v>0.41</v>
+      </c>
+      <c r="AK9">
+        <v>1.23</v>
+      </c>
+      <c r="AL9">
+        <v>1.23</v>
       </c>
       <c r="AM9">
         <v>8.77</v>
@@ -1602,7 +1740,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C10">
         <v>4.5</v>
@@ -1614,7 +1752,7 @@
         <v>-155</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G10">
         <v>823590</v>
@@ -1673,17 +1811,23 @@
       <c r="Y10">
         <v>0.9461</v>
       </c>
+      <c r="Z10">
+        <v>6</v>
+      </c>
       <c r="AA10" t="s">
         <v>44</v>
       </c>
+      <c r="AB10">
+        <v>0.21</v>
+      </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD10">
         <v>4.71</v>
       </c>
       <c r="AE10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF10">
         <v>0.2226</v>
@@ -1693,6 +1837,18 @@
       </c>
       <c r="AH10">
         <v>0</v>
+      </c>
+      <c r="AI10">
+        <v>1.29</v>
+      </c>
+      <c r="AJ10">
+        <v>1.29</v>
+      </c>
+      <c r="AK10">
+        <v>1.29</v>
+      </c>
+      <c r="AL10">
+        <v>1.29</v>
       </c>
       <c r="AM10">
         <v>4.71</v>
@@ -1703,7 +1859,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C11">
         <v>5.5</v>
@@ -1715,7 +1871,7 @@
         <v>115</v>
       </c>
       <c r="F11" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G11">
         <v>823590</v>
@@ -1774,17 +1930,23 @@
       <c r="Y11">
         <v>0.9898</v>
       </c>
+      <c r="Z11">
+        <v>7</v>
+      </c>
       <c r="AA11" t="s">
         <v>44</v>
       </c>
+      <c r="AB11">
+        <v>-0.12</v>
+      </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD11">
         <v>5.38</v>
       </c>
       <c r="AE11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF11">
         <v>0.2873</v>
@@ -1794,6 +1956,18 @@
       </c>
       <c r="AH11">
         <v>0</v>
+      </c>
+      <c r="AI11">
+        <v>1.62</v>
+      </c>
+      <c r="AJ11">
+        <v>1.62</v>
+      </c>
+      <c r="AK11">
+        <v>1.62</v>
+      </c>
+      <c r="AL11">
+        <v>1.62</v>
       </c>
       <c r="AM11">
         <v>5.38</v>
@@ -1804,7 +1978,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C12">
         <v>4.5</v>
@@ -1816,7 +1990,7 @@
         <v>-161</v>
       </c>
       <c r="F12" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G12">
         <v>824397</v>
@@ -1875,17 +2049,23 @@
       <c r="Y12">
         <v>0.88</v>
       </c>
+      <c r="Z12">
+        <v>3</v>
+      </c>
       <c r="AA12" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB12">
+        <v>-1.23</v>
       </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD12">
         <v>3.27</v>
       </c>
       <c r="AE12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF12">
         <v>0.2156</v>
@@ -1895,6 +2075,18 @@
       </c>
       <c r="AH12">
         <v>0</v>
+      </c>
+      <c r="AI12">
+        <v>-0.27</v>
+      </c>
+      <c r="AJ12">
+        <v>0.27</v>
+      </c>
+      <c r="AK12">
+        <v>-0.27</v>
+      </c>
+      <c r="AL12">
+        <v>0.27</v>
       </c>
       <c r="AM12">
         <v>3.27</v>
@@ -1905,7 +2097,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C13">
         <v>4.5</v>
@@ -1917,7 +2109,7 @@
         <v>-113</v>
       </c>
       <c r="F13" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G13">
         <v>824397</v>
@@ -1976,17 +2168,23 @@
       <c r="Y13">
         <v>1.0127</v>
       </c>
+      <c r="Z13">
+        <v>3</v>
+      </c>
       <c r="AA13" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB13">
+        <v>-0.93</v>
       </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD13">
         <v>3.57</v>
       </c>
       <c r="AE13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF13">
         <v>0.1901</v>
@@ -1996,6 +2194,18 @@
       </c>
       <c r="AH13">
         <v>0</v>
+      </c>
+      <c r="AI13">
+        <v>-0.57</v>
+      </c>
+      <c r="AJ13">
+        <v>0.57</v>
+      </c>
+      <c r="AK13">
+        <v>-0.57</v>
+      </c>
+      <c r="AL13">
+        <v>0.57</v>
       </c>
       <c r="AM13">
         <v>3.57</v>
@@ -2006,7 +2216,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C14">
         <v>5.5</v>
@@ -2018,7 +2228,7 @@
         <v>101</v>
       </c>
       <c r="F14" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G14">
         <v>824236</v>
@@ -2077,17 +2287,23 @@
       <c r="Y14">
         <v>0.88</v>
       </c>
+      <c r="Z14">
+        <v>2</v>
+      </c>
       <c r="AA14" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB14">
+        <v>-0.8</v>
       </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD14">
         <v>4.7</v>
       </c>
       <c r="AE14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF14">
         <v>0.281</v>
@@ -2097,6 +2313,18 @@
       </c>
       <c r="AH14">
         <v>0</v>
+      </c>
+      <c r="AI14">
+        <v>-2.7</v>
+      </c>
+      <c r="AJ14">
+        <v>2.7</v>
+      </c>
+      <c r="AK14">
+        <v>-2.7</v>
+      </c>
+      <c r="AL14">
+        <v>2.7</v>
       </c>
       <c r="AM14">
         <v>4.7</v>
@@ -2107,7 +2335,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C15">
         <v>4.5</v>
@@ -2119,13 +2347,13 @@
         <v>-127</v>
       </c>
       <c r="F15" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G15">
         <v>824236</v>
       </c>
       <c r="H15" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="I15">
         <v>4</v>
@@ -2178,17 +2406,23 @@
       <c r="Y15">
         <v>1.0113</v>
       </c>
+      <c r="Z15">
+        <v>5</v>
+      </c>
       <c r="AA15" t="s">
         <v>44</v>
       </c>
+      <c r="AB15">
+        <v>0.35</v>
+      </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD15">
         <v>4.85</v>
       </c>
       <c r="AE15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF15">
         <v>0.2641</v>
@@ -2198,6 +2432,18 @@
       </c>
       <c r="AH15">
         <v>0</v>
+      </c>
+      <c r="AI15">
+        <v>0.15</v>
+      </c>
+      <c r="AJ15">
+        <v>0.15</v>
+      </c>
+      <c r="AK15">
+        <v>0.15</v>
+      </c>
+      <c r="AL15">
+        <v>0.15</v>
       </c>
       <c r="AM15">
         <v>4.85</v>
@@ -2208,10 +2454,10 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F16" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G16">
         <v>824477</v>
@@ -2271,16 +2517,16 @@
         <v>1.0914</v>
       </c>
       <c r="AA16" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD16">
         <v>7.76</v>
       </c>
       <c r="AE16" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="AF16">
         <v>0.2565</v>
@@ -2300,7 +2546,7 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C17">
         <v>4.5</v>
@@ -2312,7 +2558,7 @@
         <v>100</v>
       </c>
       <c r="F17" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G17">
         <v>824477</v>
@@ -2371,17 +2617,23 @@
       <c r="Y17">
         <v>0.8813</v>
       </c>
+      <c r="Z17">
+        <v>2</v>
+      </c>
       <c r="AA17" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB17">
+        <v>-0.71</v>
       </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD17">
         <v>3.79</v>
       </c>
       <c r="AE17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF17">
         <v>0.1806</v>
@@ -2391,6 +2643,18 @@
       </c>
       <c r="AH17">
         <v>0</v>
+      </c>
+      <c r="AI17">
+        <v>-1.79</v>
+      </c>
+      <c r="AJ17">
+        <v>1.79</v>
+      </c>
+      <c r="AK17">
+        <v>-1.79</v>
+      </c>
+      <c r="AL17">
+        <v>1.79</v>
       </c>
       <c r="AM17">
         <v>3.79</v>
@@ -2401,7 +2665,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C18">
         <v>3.5</v>
@@ -2413,7 +2677,7 @@
         <v>110</v>
       </c>
       <c r="F18" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G18">
         <v>823670</v>
@@ -2472,17 +2736,23 @@
       <c r="Y18">
         <v>1</v>
       </c>
+      <c r="Z18">
+        <v>2</v>
+      </c>
       <c r="AA18" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB18">
+        <v>0.57</v>
       </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD18">
         <v>4.07</v>
       </c>
       <c r="AE18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF18">
         <v>0.1949</v>
@@ -2492,6 +2762,18 @@
       </c>
       <c r="AH18">
         <v>0</v>
+      </c>
+      <c r="AI18">
+        <v>-2.07</v>
+      </c>
+      <c r="AJ18">
+        <v>2.07</v>
+      </c>
+      <c r="AK18">
+        <v>-2.07</v>
+      </c>
+      <c r="AL18">
+        <v>2.07</v>
       </c>
       <c r="AM18">
         <v>4.07</v>
@@ -2502,7 +2784,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C19">
         <v>4.5</v>
@@ -2514,7 +2796,7 @@
         <v>-132</v>
       </c>
       <c r="F19" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G19">
         <v>823670</v>
@@ -2573,17 +2855,23 @@
       <c r="Y19">
         <v>0.9041</v>
       </c>
+      <c r="Z19">
+        <v>6</v>
+      </c>
       <c r="AA19" t="s">
         <v>44</v>
       </c>
+      <c r="AB19">
+        <v>-0.83</v>
+      </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD19">
         <v>3.67</v>
       </c>
       <c r="AE19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF19">
         <v>0.232</v>
@@ -2593,6 +2881,18 @@
       </c>
       <c r="AH19">
         <v>0</v>
+      </c>
+      <c r="AI19">
+        <v>2.33</v>
+      </c>
+      <c r="AJ19">
+        <v>2.33</v>
+      </c>
+      <c r="AK19">
+        <v>2.33</v>
+      </c>
+      <c r="AL19">
+        <v>2.33</v>
       </c>
       <c r="AM19">
         <v>3.67</v>
@@ -2603,7 +2903,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C20">
         <v>3.5</v>
@@ -2615,7 +2915,7 @@
         <v>110</v>
       </c>
       <c r="F20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G20">
         <v>824642</v>
@@ -2674,17 +2974,23 @@
       <c r="Y20">
         <v>0.9429</v>
       </c>
+      <c r="Z20">
+        <v>7</v>
+      </c>
       <c r="AA20" t="s">
         <v>44</v>
       </c>
+      <c r="AB20">
+        <v>1.54</v>
+      </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD20">
         <v>5.04</v>
       </c>
       <c r="AE20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF20">
         <v>0.2293</v>
@@ -2694,6 +3000,18 @@
       </c>
       <c r="AH20">
         <v>0</v>
+      </c>
+      <c r="AI20">
+        <v>1.96</v>
+      </c>
+      <c r="AJ20">
+        <v>1.96</v>
+      </c>
+      <c r="AK20">
+        <v>1.96</v>
+      </c>
+      <c r="AL20">
+        <v>1.96</v>
       </c>
       <c r="AM20">
         <v>5.04</v>
@@ -2704,7 +3022,7 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C21">
         <v>4.5</v>
@@ -2716,7 +3034,7 @@
         <v>-158</v>
       </c>
       <c r="F21" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G21">
         <v>824642</v>
@@ -2775,17 +3093,23 @@
       <c r="Y21">
         <v>0.915</v>
       </c>
+      <c r="Z21">
+        <v>2</v>
+      </c>
       <c r="AA21" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB21">
+        <v>-1.38</v>
       </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD21">
         <v>3.12</v>
       </c>
       <c r="AE21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF21">
         <v>0.2011</v>
@@ -2795,6 +3119,18 @@
       </c>
       <c r="AH21">
         <v>0</v>
+      </c>
+      <c r="AI21">
+        <v>-1.12</v>
+      </c>
+      <c r="AJ21">
+        <v>1.12</v>
+      </c>
+      <c r="AK21">
+        <v>-1.12</v>
+      </c>
+      <c r="AL21">
+        <v>1.12</v>
       </c>
       <c r="AM21">
         <v>3.12</v>
@@ -2805,7 +3141,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C22">
         <v>3.5</v>
@@ -2817,7 +3153,7 @@
         <v>129</v>
       </c>
       <c r="F22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="G22">
         <v>823182</v>
@@ -2876,17 +3212,23 @@
       <c r="Y22">
         <v>1.0015</v>
       </c>
+      <c r="Z22">
+        <v>2</v>
+      </c>
       <c r="AA22" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB22">
+        <v>0.68</v>
       </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD22">
         <v>4.18</v>
       </c>
       <c r="AE22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF22">
         <v>0.193</v>
@@ -2896,6 +3238,18 @@
       </c>
       <c r="AH22">
         <v>0</v>
+      </c>
+      <c r="AI22">
+        <v>-2.18</v>
+      </c>
+      <c r="AJ22">
+        <v>2.18</v>
+      </c>
+      <c r="AK22">
+        <v>-2.18</v>
+      </c>
+      <c r="AL22">
+        <v>2.18</v>
       </c>
       <c r="AM22">
         <v>4.18</v>
@@ -2906,7 +3260,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C23">
         <v>4.5</v>
@@ -2918,7 +3272,7 @@
         <v>-105</v>
       </c>
       <c r="F23" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="G23">
         <v>823182</v>
@@ -2977,17 +3331,23 @@
       <c r="Y23">
         <v>1.0278</v>
       </c>
+      <c r="Z23">
+        <v>1</v>
+      </c>
       <c r="AA23" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB23">
+        <v>0.84</v>
       </c>
       <c r="AC23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD23">
         <v>5.34</v>
       </c>
       <c r="AE23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF23">
         <v>0.1763</v>
@@ -2997,6 +3357,18 @@
       </c>
       <c r="AH23">
         <v>0</v>
+      </c>
+      <c r="AI23">
+        <v>-4.34</v>
+      </c>
+      <c r="AJ23">
+        <v>4.34</v>
+      </c>
+      <c r="AK23">
+        <v>-4.34</v>
+      </c>
+      <c r="AL23">
+        <v>4.34</v>
       </c>
       <c r="AM23">
         <v>5.34</v>
@@ -3007,7 +3379,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C24">
         <v>4.5</v>
@@ -3019,7 +3391,7 @@
         <v>-148</v>
       </c>
       <c r="F24" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G24">
         <v>824965</v>
@@ -3078,17 +3450,23 @@
       <c r="Y24">
         <v>1.0855</v>
       </c>
+      <c r="Z24">
+        <v>4</v>
+      </c>
       <c r="AA24" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB24">
+        <v>-0.97</v>
       </c>
       <c r="AC24" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD24">
         <v>3.53</v>
       </c>
       <c r="AE24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF24">
         <v>0.1538</v>
@@ -3098,6 +3476,18 @@
       </c>
       <c r="AH24">
         <v>0</v>
+      </c>
+      <c r="AI24">
+        <v>0.47</v>
+      </c>
+      <c r="AJ24">
+        <v>0.47</v>
+      </c>
+      <c r="AK24">
+        <v>0.47</v>
+      </c>
+      <c r="AL24">
+        <v>0.47</v>
       </c>
       <c r="AM24">
         <v>3.53</v>
@@ -3108,7 +3498,7 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C25">
         <v>4.5</v>
@@ -3120,7 +3510,7 @@
         <v>112</v>
       </c>
       <c r="F25" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G25">
         <v>824965</v>
@@ -3179,17 +3569,23 @@
       <c r="Y25">
         <v>1.0819</v>
       </c>
+      <c r="Z25">
+        <v>6</v>
+      </c>
       <c r="AA25" t="s">
         <v>44</v>
       </c>
+      <c r="AB25">
+        <v>0.95</v>
+      </c>
       <c r="AC25" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD25">
         <v>5.45</v>
       </c>
       <c r="AE25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF25">
         <v>0.2317</v>
@@ -3199,6 +3595,18 @@
       </c>
       <c r="AH25">
         <v>0</v>
+      </c>
+      <c r="AI25">
+        <v>0.55</v>
+      </c>
+      <c r="AJ25">
+        <v>0.55</v>
+      </c>
+      <c r="AK25">
+        <v>0.55</v>
+      </c>
+      <c r="AL25">
+        <v>0.55</v>
       </c>
       <c r="AM25">
         <v>5.45</v>
@@ -3209,7 +3617,7 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C26">
         <v>5.5</v>
@@ -3221,7 +3629,7 @@
         <v>128</v>
       </c>
       <c r="F26" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="G26">
         <v>823991</v>
@@ -3280,17 +3688,23 @@
       <c r="Y26">
         <v>1.0952</v>
       </c>
+      <c r="Z26">
+        <v>8</v>
+      </c>
       <c r="AA26" t="s">
         <v>44</v>
       </c>
+      <c r="AB26">
+        <v>1.43</v>
+      </c>
       <c r="AC26" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD26">
         <v>6.93</v>
       </c>
       <c r="AE26" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="AF26">
         <v>0.1996</v>
@@ -3300,6 +3714,18 @@
       </c>
       <c r="AH26">
         <v>0</v>
+      </c>
+      <c r="AI26">
+        <v>1.07</v>
+      </c>
+      <c r="AJ26">
+        <v>1.07</v>
+      </c>
+      <c r="AK26">
+        <v>1.07</v>
+      </c>
+      <c r="AL26">
+        <v>1.07</v>
       </c>
       <c r="AM26">
         <v>6.93</v>
@@ -3310,7 +3736,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C27">
         <v>3.5</v>
@@ -3322,7 +3748,7 @@
         <v>131</v>
       </c>
       <c r="F27" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="G27">
         <v>823991</v>
@@ -3381,17 +3807,23 @@
       <c r="Y27">
         <v>1.0004</v>
       </c>
+      <c r="Z27">
+        <v>4</v>
+      </c>
       <c r="AA27" t="s">
         <v>44</v>
       </c>
+      <c r="AB27">
+        <v>-0.28</v>
+      </c>
       <c r="AC27" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD27">
         <v>3.22</v>
       </c>
       <c r="AE27" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF27">
         <v>0.1711</v>
@@ -3401,6 +3833,18 @@
       </c>
       <c r="AH27">
         <v>0</v>
+      </c>
+      <c r="AI27">
+        <v>0.78</v>
+      </c>
+      <c r="AJ27">
+        <v>0.78</v>
+      </c>
+      <c r="AK27">
+        <v>0.78</v>
+      </c>
+      <c r="AL27">
+        <v>0.78</v>
       </c>
       <c r="AM27">
         <v>3.22</v>
@@ -3411,7 +3855,7 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C28">
         <v>5.5</v>
@@ -3423,7 +3867,7 @@
         <v>-120</v>
       </c>
       <c r="F28" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G28">
         <v>823912</v>
@@ -3482,17 +3926,23 @@
       <c r="Y28">
         <v>0.9497</v>
       </c>
+      <c r="Z28">
+        <v>6</v>
+      </c>
       <c r="AA28" t="s">
         <v>44</v>
       </c>
+      <c r="AB28">
+        <v>0.41</v>
+      </c>
       <c r="AC28" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD28">
         <v>5.91</v>
       </c>
       <c r="AE28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF28">
         <v>0.3252</v>
@@ -3502,6 +3952,18 @@
       </c>
       <c r="AH28">
         <v>0</v>
+      </c>
+      <c r="AI28">
+        <v>0.09</v>
+      </c>
+      <c r="AJ28">
+        <v>0.09</v>
+      </c>
+      <c r="AK28">
+        <v>0.09</v>
+      </c>
+      <c r="AL28">
+        <v>0.09</v>
       </c>
       <c r="AM28">
         <v>5.91</v>
@@ -3512,7 +3974,7 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C29">
         <v>7.5</v>
@@ -3524,7 +3986,7 @@
         <v>-136</v>
       </c>
       <c r="F29" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G29">
         <v>823912</v>
@@ -3583,17 +4045,23 @@
       <c r="Y29">
         <v>0.9968</v>
       </c>
+      <c r="Z29">
+        <v>7</v>
+      </c>
       <c r="AA29" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB29">
+        <v>0.24</v>
       </c>
       <c r="AC29" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD29">
         <v>8.56</v>
       </c>
       <c r="AE29" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="AF29">
         <v>0.2916</v>
@@ -3603,6 +4071,18 @@
       </c>
       <c r="AH29">
         <v>-0.82</v>
+      </c>
+      <c r="AI29">
+        <v>-1.56</v>
+      </c>
+      <c r="AJ29">
+        <v>1.56</v>
+      </c>
+      <c r="AK29">
+        <v>-0.74</v>
+      </c>
+      <c r="AL29">
+        <v>0.74</v>
       </c>
       <c r="AM29">
         <v>7.74</v>
@@ -3613,7 +4093,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C30">
         <v>5.5</v>
@@ -3625,7 +4105,7 @@
         <v>-104</v>
       </c>
       <c r="F30" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G30">
         <v>824156</v>
@@ -3684,17 +4164,23 @@
       <c r="Y30">
         <v>0.9454</v>
       </c>
+      <c r="Z30">
+        <v>4</v>
+      </c>
       <c r="AA30" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB30">
+        <v>-1.54</v>
       </c>
       <c r="AC30" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD30">
         <v>3.96</v>
       </c>
       <c r="AE30" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF30">
         <v>0.2486</v>
@@ -3704,6 +4190,18 @@
       </c>
       <c r="AH30">
         <v>0</v>
+      </c>
+      <c r="AI30">
+        <v>0.04</v>
+      </c>
+      <c r="AJ30">
+        <v>0.04</v>
+      </c>
+      <c r="AK30">
+        <v>0.04</v>
+      </c>
+      <c r="AL30">
+        <v>0.04</v>
       </c>
       <c r="AM30">
         <v>3.96</v>
@@ -3714,7 +4212,7 @@
         <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C31">
         <v>5.5</v>
@@ -3726,7 +4224,7 @@
         <v>-102</v>
       </c>
       <c r="F31" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G31">
         <v>824156</v>
@@ -3785,17 +4283,23 @@
       <c r="Y31">
         <v>1.006</v>
       </c>
+      <c r="Z31">
+        <v>5</v>
+      </c>
       <c r="AA31" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB31">
+        <v>0.14</v>
       </c>
       <c r="AC31" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AD31">
         <v>5.64</v>
       </c>
       <c r="AE31" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF31">
         <v>0.2462</v>
@@ -3805,6 +4309,18 @@
       </c>
       <c r="AH31">
         <v>0</v>
+      </c>
+      <c r="AI31">
+        <v>-0.64</v>
+      </c>
+      <c r="AJ31">
+        <v>0.64</v>
+      </c>
+      <c r="AK31">
+        <v>-0.64</v>
+      </c>
+      <c r="AL31">
+        <v>0.64</v>
       </c>
       <c r="AM31">
         <v>5.64</v>
@@ -3815,7 +4331,7 @@
         <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C32">
         <v>6.5</v>
@@ -3827,31 +4343,31 @@
         <v>-105</v>
       </c>
       <c r="F32" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G32" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="H32" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="L32">
         <v>6</v>
       </c>
       <c r="S32" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="V32" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AA32" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AC32" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="AE32" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>